<commit_message>
cambio visual en controles, plan de parto y riesgo
</commit_message>
<xml_diff>
--- a/backend/src/assets/official_forms/plan_parto_oficial.xlsx
+++ b/backend/src/assets/official_forms/plan_parto_oficial.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94E2CA7A-A4C3-4B2A-991E-00597C2123FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A4025DA-D11A-4525-8D2F-C74A9F587A95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="plan de parto" sheetId="1" r:id="rId1"/>
@@ -990,7 +990,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="118">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1131,6 +1131,69 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="justify"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1152,68 +1215,11 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="justify"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1600,43 +1606,43 @@
       <c r="C3" s="6"/>
       <c r="D3" s="6"/>
       <c r="E3" s="7"/>
-      <c r="F3" s="90" t="s">
+      <c r="F3" s="111" t="s">
         <v>2</v>
       </c>
-      <c r="G3" s="91"/>
-      <c r="H3" s="91"/>
-      <c r="I3" s="91"/>
-      <c r="J3" s="91"/>
-      <c r="K3" s="91"/>
-      <c r="L3" s="91"/>
-      <c r="M3" s="91"/>
-      <c r="N3" s="91"/>
-      <c r="O3" s="91"/>
-      <c r="P3" s="91"/>
-      <c r="Q3" s="91"/>
-      <c r="R3" s="91"/>
-      <c r="S3" s="91"/>
-      <c r="T3" s="91"/>
-      <c r="U3" s="92"/>
-      <c r="W3" s="96" t="s">
+      <c r="G3" s="112"/>
+      <c r="H3" s="112"/>
+      <c r="I3" s="112"/>
+      <c r="J3" s="112"/>
+      <c r="K3" s="112"/>
+      <c r="L3" s="112"/>
+      <c r="M3" s="112"/>
+      <c r="N3" s="112"/>
+      <c r="O3" s="112"/>
+      <c r="P3" s="112"/>
+      <c r="Q3" s="112"/>
+      <c r="R3" s="112"/>
+      <c r="S3" s="112"/>
+      <c r="T3" s="112"/>
+      <c r="U3" s="113"/>
+      <c r="W3" s="117" t="s">
         <v>3</v>
       </c>
-      <c r="X3" s="96"/>
-      <c r="Y3" s="97"/>
-      <c r="Z3" s="97"/>
-      <c r="AA3" s="97"/>
-      <c r="AB3" s="97"/>
-      <c r="AC3" s="99"/>
-      <c r="AD3" s="97"/>
-      <c r="AE3" s="97"/>
-      <c r="AF3" s="97"/>
-      <c r="AG3" s="101"/>
-      <c r="AH3" s="97"/>
-      <c r="AI3" s="99"/>
-      <c r="AJ3" s="97"/>
-      <c r="AK3" s="97"/>
-      <c r="AL3" s="97"/>
-      <c r="AM3" s="97"/>
+      <c r="X3" s="117"/>
+      <c r="Y3" s="99"/>
+      <c r="Z3" s="99"/>
+      <c r="AA3" s="99"/>
+      <c r="AB3" s="99"/>
+      <c r="AC3" s="109"/>
+      <c r="AD3" s="99"/>
+      <c r="AE3" s="99"/>
+      <c r="AF3" s="99"/>
+      <c r="AG3" s="108"/>
+      <c r="AH3" s="99"/>
+      <c r="AI3" s="109"/>
+      <c r="AJ3" s="99"/>
+      <c r="AK3" s="99"/>
+      <c r="AL3" s="99"/>
+      <c r="AM3" s="99"/>
       <c r="AN3" s="8"/>
     </row>
     <row r="4" spans="1:49" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1645,40 +1651,40 @@
       <c r="C4" s="10"/>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
-      <c r="F4" s="93"/>
-      <c r="G4" s="94"/>
-      <c r="H4" s="94"/>
-      <c r="I4" s="94"/>
-      <c r="J4" s="94"/>
-      <c r="K4" s="94"/>
-      <c r="L4" s="94"/>
-      <c r="M4" s="94"/>
-      <c r="N4" s="94"/>
-      <c r="O4" s="94"/>
-      <c r="P4" s="94"/>
-      <c r="Q4" s="94"/>
-      <c r="R4" s="94"/>
-      <c r="S4" s="94"/>
-      <c r="T4" s="94"/>
-      <c r="U4" s="95"/>
+      <c r="F4" s="114"/>
+      <c r="G4" s="115"/>
+      <c r="H4" s="115"/>
+      <c r="I4" s="115"/>
+      <c r="J4" s="115"/>
+      <c r="K4" s="115"/>
+      <c r="L4" s="115"/>
+      <c r="M4" s="115"/>
+      <c r="N4" s="115"/>
+      <c r="O4" s="115"/>
+      <c r="P4" s="115"/>
+      <c r="Q4" s="115"/>
+      <c r="R4" s="115"/>
+      <c r="S4" s="115"/>
+      <c r="T4" s="115"/>
+      <c r="U4" s="116"/>
       <c r="V4" s="11"/>
-      <c r="W4" s="96"/>
-      <c r="X4" s="96"/>
-      <c r="Y4" s="98"/>
-      <c r="Z4" s="98"/>
-      <c r="AA4" s="98"/>
-      <c r="AB4" s="98"/>
-      <c r="AC4" s="100"/>
-      <c r="AD4" s="98"/>
-      <c r="AE4" s="98"/>
-      <c r="AF4" s="98"/>
-      <c r="AG4" s="101"/>
-      <c r="AH4" s="98"/>
-      <c r="AI4" s="100"/>
-      <c r="AJ4" s="98"/>
-      <c r="AK4" s="98"/>
-      <c r="AL4" s="98"/>
-      <c r="AM4" s="97"/>
+      <c r="W4" s="117"/>
+      <c r="X4" s="117"/>
+      <c r="Y4" s="100"/>
+      <c r="Z4" s="100"/>
+      <c r="AA4" s="100"/>
+      <c r="AB4" s="100"/>
+      <c r="AC4" s="110"/>
+      <c r="AD4" s="100"/>
+      <c r="AE4" s="100"/>
+      <c r="AF4" s="100"/>
+      <c r="AG4" s="108"/>
+      <c r="AH4" s="100"/>
+      <c r="AI4" s="110"/>
+      <c r="AJ4" s="100"/>
+      <c r="AK4" s="100"/>
+      <c r="AL4" s="100"/>
+      <c r="AM4" s="99"/>
       <c r="AN4" s="12"/>
     </row>
     <row r="5" spans="1:49" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1710,20 +1716,20 @@
       <c r="X5" s="17"/>
       <c r="Y5" s="16"/>
       <c r="Z5" s="16"/>
-      <c r="AA5" s="16"/>
-      <c r="AB5" s="16"/>
-      <c r="AC5" s="16"/>
-      <c r="AD5" s="16"/>
-      <c r="AE5" s="16"/>
-      <c r="AF5" s="16"/>
-      <c r="AG5" s="16"/>
-      <c r="AH5" s="16"/>
-      <c r="AI5" s="16"/>
-      <c r="AJ5" s="16"/>
-      <c r="AK5" s="16"/>
-      <c r="AL5" s="16"/>
-      <c r="AM5" s="16"/>
-      <c r="AN5" s="18"/>
+      <c r="AA5" s="118"/>
+      <c r="AB5" s="118"/>
+      <c r="AC5" s="118"/>
+      <c r="AD5" s="118"/>
+      <c r="AE5" s="118"/>
+      <c r="AF5" s="118"/>
+      <c r="AG5" s="118"/>
+      <c r="AH5" s="118"/>
+      <c r="AI5" s="118"/>
+      <c r="AJ5" s="118"/>
+      <c r="AK5" s="118"/>
+      <c r="AL5" s="118"/>
+      <c r="AM5" s="118"/>
+      <c r="AN5" s="119"/>
       <c r="AO5" s="14"/>
       <c r="AW5" s="19"/>
     </row>
@@ -1849,16 +1855,16 @@
       <c r="AB8" s="17"/>
       <c r="AC8" s="17"/>
       <c r="AD8" s="17"/>
-      <c r="AE8" s="116"/>
-      <c r="AF8" s="116"/>
-      <c r="AG8" s="116"/>
-      <c r="AH8" s="116"/>
-      <c r="AI8" s="116"/>
-      <c r="AJ8" s="116"/>
-      <c r="AK8" s="116"/>
-      <c r="AL8" s="116"/>
-      <c r="AM8" s="116"/>
-      <c r="AN8" s="117"/>
+      <c r="AE8" s="106"/>
+      <c r="AF8" s="106"/>
+      <c r="AG8" s="106"/>
+      <c r="AH8" s="106"/>
+      <c r="AI8" s="106"/>
+      <c r="AJ8" s="106"/>
+      <c r="AK8" s="106"/>
+      <c r="AL8" s="106"/>
+      <c r="AM8" s="106"/>
+      <c r="AN8" s="107"/>
       <c r="AO8" s="14"/>
     </row>
     <row r="9" spans="1:49" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1975,8 +1981,8 @@
       <c r="S11" s="17"/>
       <c r="T11" s="17"/>
       <c r="U11" s="17"/>
-      <c r="V11" s="102"/>
-      <c r="W11" s="105"/>
+      <c r="V11" s="101"/>
+      <c r="W11" s="104"/>
       <c r="X11" s="22"/>
       <c r="Y11" s="26" t="s">
         <v>15</v>
@@ -2036,8 +2042,8 @@
       </c>
       <c r="T12" s="35"/>
       <c r="U12" s="19"/>
-      <c r="V12" s="103"/>
-      <c r="W12" s="106"/>
+      <c r="V12" s="102"/>
+      <c r="W12" s="105"/>
       <c r="X12" s="37" t="s">
         <v>23</v>
       </c>
@@ -2087,8 +2093,8 @@
       <c r="S13" s="19"/>
       <c r="T13" s="19"/>
       <c r="U13" s="19"/>
-      <c r="V13" s="103"/>
-      <c r="W13" s="106"/>
+      <c r="V13" s="102"/>
+      <c r="W13" s="105"/>
       <c r="X13" s="13"/>
       <c r="Y13" s="14"/>
       <c r="Z13" s="14"/>
@@ -2140,8 +2146,8 @@
       <c r="S14" s="39"/>
       <c r="T14" s="39"/>
       <c r="U14" s="39"/>
-      <c r="V14" s="104"/>
-      <c r="W14" s="106"/>
+      <c r="V14" s="103"/>
+      <c r="W14" s="105"/>
       <c r="X14" s="13" t="s">
         <v>32</v>
       </c>
@@ -2192,7 +2198,7 @@
       <c r="T15" s="14"/>
       <c r="U15" s="14"/>
       <c r="V15" s="14"/>
-      <c r="W15" s="106"/>
+      <c r="W15" s="105"/>
       <c r="X15" s="13"/>
       <c r="Y15" s="14"/>
       <c r="Z15" s="14"/>
@@ -2309,7 +2315,7 @@
       <c r="AO17" s="14"/>
     </row>
     <row r="18" spans="1:41" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="107" t="s">
+      <c r="A18" s="90" t="s">
         <v>41</v>
       </c>
       <c r="B18" s="36"/>
@@ -2364,7 +2370,7 @@
       <c r="AO18" s="14"/>
     </row>
     <row r="19" spans="1:41" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="108"/>
+      <c r="A19" s="91"/>
       <c r="B19" s="36"/>
       <c r="C19" s="14" t="s">
         <v>47</v>
@@ -2414,7 +2420,7 @@
       <c r="AO19" s="14"/>
     </row>
     <row r="20" spans="1:41" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="108"/>
+      <c r="A20" s="91"/>
       <c r="B20" s="36"/>
       <c r="C20" s="14" t="s">
         <v>51</v>
@@ -2461,7 +2467,7 @@
       <c r="AO20" s="14"/>
     </row>
     <row r="21" spans="1:41" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="108"/>
+      <c r="A21" s="91"/>
       <c r="B21" s="36"/>
       <c r="I21" s="14"/>
       <c r="J21" s="14"/>
@@ -2488,7 +2494,7 @@
       <c r="AO21" s="14"/>
     </row>
     <row r="22" spans="1:41" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="108"/>
+      <c r="A22" s="91"/>
       <c r="B22" s="36"/>
       <c r="C22" s="14" t="s">
         <v>53</v>
@@ -2540,7 +2546,7 @@
       <c r="AO22" s="14"/>
     </row>
     <row r="23" spans="1:41" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="108"/>
+      <c r="A23" s="91"/>
       <c r="B23" s="36"/>
       <c r="C23" s="14"/>
       <c r="D23" s="14"/>
@@ -2575,7 +2581,7 @@
       <c r="AO23" s="14"/>
     </row>
     <row r="24" spans="1:41" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="108"/>
+      <c r="A24" s="91"/>
       <c r="B24" s="36"/>
       <c r="C24" s="3" t="s">
         <v>59</v>
@@ -2623,7 +2629,7 @@
       <c r="AO24" s="14"/>
     </row>
     <row r="25" spans="1:41" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="108"/>
+      <c r="A25" s="91"/>
       <c r="B25" s="36"/>
       <c r="C25" s="3" t="s">
         <v>60</v>
@@ -2673,7 +2679,7 @@
       <c r="AO25" s="14"/>
     </row>
     <row r="26" spans="1:41" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="108"/>
+      <c r="A26" s="91"/>
       <c r="B26" s="36"/>
       <c r="C26" s="3" t="s">
         <v>64</v>
@@ -2723,7 +2729,7 @@
       <c r="AO26" s="14"/>
     </row>
     <row r="27" spans="1:41" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="108"/>
+      <c r="A27" s="91"/>
       <c r="B27" s="36"/>
       <c r="C27" s="19"/>
       <c r="D27" s="19"/>
@@ -2771,7 +2777,7 @@
       <c r="AO27" s="14"/>
     </row>
     <row r="28" spans="1:41" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="108"/>
+      <c r="A28" s="91"/>
       <c r="B28" s="36"/>
       <c r="C28" s="14"/>
       <c r="D28" s="14"/>
@@ -2819,7 +2825,7 @@
       <c r="AO28" s="14"/>
     </row>
     <row r="29" spans="1:41" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="108"/>
+      <c r="A29" s="91"/>
       <c r="B29" s="14"/>
       <c r="AN29" s="54"/>
       <c r="AO29" s="14"/>
@@ -4274,11 +4280,11 @@
       <c r="AO62" s="14"/>
     </row>
     <row r="63" spans="1:62" ht="9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="109" t="s">
+      <c r="A63" s="92" t="s">
         <v>138</v>
       </c>
-      <c r="B63" s="110"/>
-      <c r="C63" s="110"/>
+      <c r="B63" s="93"/>
+      <c r="C63" s="93"/>
       <c r="D63" s="77"/>
       <c r="E63" s="77"/>
       <c r="F63" s="77"/>
@@ -4321,11 +4327,11 @@
       <c r="AO63" s="14"/>
     </row>
     <row r="64" spans="1:62" ht="9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="111" t="s">
+      <c r="A64" s="94" t="s">
         <v>139</v>
       </c>
-      <c r="B64" s="112"/>
-      <c r="C64" s="112"/>
+      <c r="B64" s="95"/>
+      <c r="C64" s="95"/>
       <c r="D64" s="80"/>
       <c r="E64" s="80"/>
       <c r="F64" s="80"/>
@@ -4367,11 +4373,11 @@
       <c r="AO64" s="14"/>
     </row>
     <row r="65" spans="1:41" ht="9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="111" t="s">
+      <c r="A65" s="94" t="s">
         <v>141</v>
       </c>
-      <c r="B65" s="112"/>
-      <c r="C65" s="112"/>
+      <c r="B65" s="95"/>
+      <c r="C65" s="95"/>
       <c r="D65" s="80"/>
       <c r="E65" s="80"/>
       <c r="F65" s="80"/>
@@ -4663,39 +4669,39 @@
       <c r="AO71" s="14"/>
     </row>
     <row r="72" spans="1:41" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="113" t="s">
+      <c r="A72" s="96" t="s">
         <v>144</v>
       </c>
-      <c r="B72" s="114"/>
-      <c r="C72" s="114"/>
-      <c r="D72" s="114"/>
-      <c r="E72" s="114"/>
-      <c r="F72" s="114"/>
-      <c r="G72" s="114"/>
-      <c r="H72" s="114"/>
-      <c r="I72" s="114"/>
-      <c r="J72" s="114"/>
-      <c r="K72" s="114"/>
-      <c r="L72" s="114"/>
-      <c r="M72" s="114"/>
-      <c r="N72" s="114"/>
-      <c r="O72" s="114"/>
-      <c r="P72" s="114"/>
-      <c r="Q72" s="114"/>
-      <c r="R72" s="114"/>
-      <c r="S72" s="114"/>
-      <c r="T72" s="114"/>
-      <c r="U72" s="114"/>
-      <c r="V72" s="114"/>
-      <c r="W72" s="114"/>
-      <c r="X72" s="114"/>
-      <c r="Y72" s="114"/>
-      <c r="Z72" s="114"/>
-      <c r="AA72" s="114"/>
-      <c r="AB72" s="114"/>
-      <c r="AC72" s="114"/>
-      <c r="AD72" s="114"/>
-      <c r="AE72" s="115"/>
+      <c r="B72" s="97"/>
+      <c r="C72" s="97"/>
+      <c r="D72" s="97"/>
+      <c r="E72" s="97"/>
+      <c r="F72" s="97"/>
+      <c r="G72" s="97"/>
+      <c r="H72" s="97"/>
+      <c r="I72" s="97"/>
+      <c r="J72" s="97"/>
+      <c r="K72" s="97"/>
+      <c r="L72" s="97"/>
+      <c r="M72" s="97"/>
+      <c r="N72" s="97"/>
+      <c r="O72" s="97"/>
+      <c r="P72" s="97"/>
+      <c r="Q72" s="97"/>
+      <c r="R72" s="97"/>
+      <c r="S72" s="97"/>
+      <c r="T72" s="97"/>
+      <c r="U72" s="97"/>
+      <c r="V72" s="97"/>
+      <c r="W72" s="97"/>
+      <c r="X72" s="97"/>
+      <c r="Y72" s="97"/>
+      <c r="Z72" s="97"/>
+      <c r="AA72" s="97"/>
+      <c r="AB72" s="97"/>
+      <c r="AC72" s="97"/>
+      <c r="AD72" s="97"/>
+      <c r="AE72" s="98"/>
       <c r="AG72" s="33" t="s">
         <v>145</v>
       </c>
@@ -4778,12 +4784,13 @@
       <c r="AO74" s="19"/>
     </row>
   </sheetData>
-  <mergeCells count="26">
-    <mergeCell ref="A18:A29"/>
-    <mergeCell ref="A63:C63"/>
-    <mergeCell ref="A64:C64"/>
-    <mergeCell ref="A65:C65"/>
-    <mergeCell ref="A72:AE72"/>
+  <mergeCells count="27">
+    <mergeCell ref="AA5:AN5"/>
+    <mergeCell ref="F3:U4"/>
+    <mergeCell ref="W3:X4"/>
+    <mergeCell ref="Y3:Y4"/>
+    <mergeCell ref="Z3:Z4"/>
+    <mergeCell ref="AA3:AA4"/>
     <mergeCell ref="AL3:AL4"/>
     <mergeCell ref="AM3:AM4"/>
     <mergeCell ref="V11:V14"/>
@@ -4800,11 +4807,11 @@
     <mergeCell ref="AD3:AD4"/>
     <mergeCell ref="AE3:AE4"/>
     <mergeCell ref="AF3:AF4"/>
-    <mergeCell ref="F3:U4"/>
-    <mergeCell ref="W3:X4"/>
-    <mergeCell ref="Y3:Y4"/>
-    <mergeCell ref="Z3:Z4"/>
-    <mergeCell ref="AA3:AA4"/>
+    <mergeCell ref="A18:A29"/>
+    <mergeCell ref="A63:C63"/>
+    <mergeCell ref="A64:C64"/>
+    <mergeCell ref="A65:C65"/>
+    <mergeCell ref="A72:AE72"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.11811023622047245" right="0" top="0" bottom="0" header="0.11811023622047245" footer="0.11811023622047245"/>

</xml_diff>